<commit_message>
chore: monthly data update 2026-05
</commit_message>
<xml_diff>
--- a/data/processed/salary_tracker_uk.xlsx
+++ b/data/processed/salary_tracker_uk.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -438,46 +438,57 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>2023</v>
+        <v>2019</v>
       </c>
       <c r="B2" t="n">
-        <v>3750</v>
+        <v>3083</v>
       </c>
       <c r="C2" t="n">
-        <v>45000</v>
+        <v>37000</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2024</v>
+        <v>2020</v>
       </c>
       <c r="B3" t="n">
-        <v>3875</v>
+        <v>3167</v>
       </c>
       <c r="C3" t="n">
-        <v>46500</v>
+        <v>38000</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>2025</v>
+        <v>2021</v>
       </c>
       <c r="B4" t="n">
-        <v>4000</v>
+        <v>3500</v>
       </c>
       <c r="C4" t="n">
-        <v>48000</v>
+        <v>42000</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>2026</v>
+        <v>2022</v>
       </c>
       <c r="B5" t="n">
-        <v>4167</v>
+        <v>3750</v>
       </c>
       <c r="C5" t="n">
-        <v>50000</v>
+        <v>45000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B6" t="n">
+        <v>5167</v>
+      </c>
+      <c r="C6" t="n">
+        <v>62000</v>
       </c>
     </row>
   </sheetData>
@@ -5107,7 +5118,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5184,43 +5195,43 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>2023</v>
+        <v>2019</v>
       </c>
       <c r="B2" t="n">
-        <v>3750</v>
+        <v>3083</v>
       </c>
       <c r="C2" t="n">
-        <v>45000</v>
+        <v>37000</v>
       </c>
       <c r="D2" t="n">
-        <v>23.08</v>
+        <v>18.97</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>-40.32</v>
       </c>
       <c r="F2" t="n">
-        <v>130.54</v>
+        <v>107.8</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>-17.42</v>
       </c>
       <c r="H2" t="n">
-        <v>45000</v>
+        <v>44805.58</v>
       </c>
       <c r="I2" t="n">
-        <v>3750</v>
+        <v>3733.39</v>
       </c>
       <c r="J2" t="n">
-        <v>23.08</v>
+        <v>22.98</v>
       </c>
       <c r="K2" t="n">
-        <v>0</v>
+        <v>-27.73</v>
       </c>
       <c r="L2" t="n">
-        <v>0</v>
+        <v>-17194.42</v>
       </c>
       <c r="M2" t="n">
-        <v>0</v>
+        <v>-1433.61</v>
       </c>
       <c r="N2" t="n">
         <v/>
@@ -5228,134 +5239,178 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2024</v>
+        <v>2020</v>
       </c>
       <c r="B3" t="n">
-        <v>3875</v>
+        <v>3167</v>
       </c>
       <c r="C3" t="n">
-        <v>46500</v>
+        <v>38000</v>
       </c>
       <c r="D3" t="n">
-        <v>23.85</v>
+        <v>19.49</v>
       </c>
       <c r="E3" t="n">
-        <v>3.33</v>
+        <v>-38.71</v>
       </c>
       <c r="F3" t="n">
-        <v>133.86</v>
+        <v>108.75</v>
       </c>
       <c r="G3" t="n">
-        <v>2.54</v>
+        <v>-16.69</v>
       </c>
       <c r="H3" t="n">
-        <v>45347.85</v>
+        <v>45614.56</v>
       </c>
       <c r="I3" t="n">
-        <v>3778.99</v>
+        <v>3801.61</v>
       </c>
       <c r="J3" t="n">
-        <v>23.26</v>
+        <v>23.39</v>
       </c>
       <c r="K3" t="n">
-        <v>0.77</v>
+        <v>-26.43</v>
       </c>
       <c r="L3" t="n">
-        <v>347.85</v>
+        <v>-16385.44</v>
       </c>
       <c r="M3" t="n">
-        <v>28.99</v>
+        <v>-1365.39</v>
       </c>
       <c r="N3" t="n">
-        <v>0.77</v>
+        <v>1.81</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>2025</v>
+        <v>2021</v>
       </c>
       <c r="B4" t="n">
-        <v>4000</v>
+        <v>3500</v>
       </c>
       <c r="C4" t="n">
-        <v>48000</v>
+        <v>42000</v>
       </c>
       <c r="D4" t="n">
-        <v>24.62</v>
+        <v>21.54</v>
       </c>
       <c r="E4" t="n">
-        <v>6.67</v>
+        <v>-32.26</v>
       </c>
       <c r="F4" t="n">
-        <v>138.37</v>
+        <v>111.56</v>
       </c>
       <c r="G4" t="n">
-        <v>5.99</v>
+        <v>-14.54</v>
       </c>
       <c r="H4" t="n">
-        <v>45285.47</v>
+        <v>49146.93</v>
       </c>
       <c r="I4" t="n">
-        <v>3773.79</v>
+        <v>4095.58</v>
       </c>
       <c r="J4" t="n">
-        <v>23.22</v>
+        <v>25.2</v>
       </c>
       <c r="K4" t="n">
-        <v>0.63</v>
+        <v>-20.73</v>
       </c>
       <c r="L4" t="n">
-        <v>285.47</v>
+        <v>-12853.07</v>
       </c>
       <c r="M4" t="n">
-        <v>23.79</v>
+        <v>-1071.42</v>
       </c>
       <c r="N4" t="n">
-        <v>-0.14</v>
+        <v>7.74</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>2026</v>
+        <v>2022</v>
       </c>
       <c r="B5" t="n">
-        <v>4167</v>
+        <v>3750</v>
       </c>
       <c r="C5" t="n">
-        <v>50000</v>
+        <v>45000</v>
       </c>
       <c r="D5" t="n">
-        <v>25.64</v>
+        <v>23.08</v>
       </c>
       <c r="E5" t="n">
-        <v>11.11</v>
+        <v>-27.42</v>
       </c>
       <c r="F5" t="n">
-        <v>140.2</v>
+        <v>121.66</v>
       </c>
       <c r="G5" t="n">
-        <v>7.4</v>
+        <v>-6.8</v>
       </c>
       <c r="H5" t="n">
-        <v>46555.52</v>
+        <v>48285.84</v>
       </c>
       <c r="I5" t="n">
-        <v>3879.94</v>
+        <v>4023.82</v>
       </c>
       <c r="J5" t="n">
-        <v>23.87</v>
+        <v>24.76</v>
       </c>
       <c r="K5" t="n">
-        <v>3.46</v>
+        <v>-22.12</v>
       </c>
       <c r="L5" t="n">
-        <v>1555.52</v>
+        <v>-13714.16</v>
       </c>
       <c r="M5" t="n">
-        <v>129.94</v>
+        <v>-1143.18</v>
       </c>
       <c r="N5" t="n">
-        <v>2.8</v>
+        <v>-1.75</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B6" t="n">
+        <v>5167</v>
+      </c>
+      <c r="C6" t="n">
+        <v>62000</v>
+      </c>
+      <c r="D6" t="n">
+        <v>31.79</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>130.54</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>62000</v>
+      </c>
+      <c r="I6" t="n">
+        <v>5167</v>
+      </c>
+      <c r="J6" t="n">
+        <v>31.79</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" t="n">
+        <v>28.4</v>
       </c>
     </row>
   </sheetData>
@@ -5453,7 +5508,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>2026</v>
+        <v>2023</v>
       </c>
     </row>
     <row r="9">
@@ -5463,7 +5518,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>4167</v>
+        <v>5167</v>
       </c>
     </row>
     <row r="10">
@@ -5473,7 +5528,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>50000</v>
+        <v>62000</v>
       </c>
     </row>
     <row r="11">
@@ -5483,7 +5538,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>25.64</v>
+        <v>31.79</v>
       </c>
     </row>
     <row r="12">
@@ -5493,7 +5548,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>3857.92</v>
+        <v>4783.75</v>
       </c>
     </row>
     <row r="13">
@@ -5503,7 +5558,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>46291.37</v>
+        <v>57401.3</v>
       </c>
     </row>
     <row r="14">
@@ -5513,7 +5568,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>23.74</v>
+        <v>29.44</v>
       </c>
     </row>
     <row r="15">
@@ -5533,7 +5588,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>11.11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -5543,7 +5598,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>2.87</v>
+        <v>-7.42</v>
       </c>
     </row>
     <row r="18">
@@ -5553,7 +5608,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>1291.37</v>
+        <v>-4598.7</v>
       </c>
     </row>
     <row r="19">
@@ -5563,7 +5618,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>107.92</v>
+        <v>-383.25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: monthly data update 2026-06
</commit_message>
<xml_diff>
--- a/data/processed/salary_tracker_uk.xlsx
+++ b/data/processed/salary_tracker_uk.xlsx
@@ -502,7 +502,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B460"/>
+  <dimension ref="A1:B461"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5105,6 +5105,16 @@
       </c>
       <c r="B460" t="n">
         <v>141</v>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B461" t="n">
+        <v>142.1</v>
       </c>
     </row>
   </sheetData>
@@ -5447,7 +5457,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-04</t>
         </is>
       </c>
     </row>
@@ -5458,7 +5468,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>141</v>
+        <v>142.1</v>
       </c>
     </row>
     <row r="4">
@@ -5548,7 +5558,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>4783.75</v>
+        <v>4746.72</v>
       </c>
     </row>
     <row r="13">
@@ -5558,7 +5568,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>57401.3</v>
+        <v>56956.96</v>
       </c>
     </row>
     <row r="14">
@@ -5568,7 +5578,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>29.44</v>
+        <v>29.21</v>
       </c>
     </row>
     <row r="15">
@@ -5578,7 +5588,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>8.01</v>
+        <v>8.85</v>
       </c>
     </row>
     <row r="16">
@@ -5598,7 +5608,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>-7.42</v>
+        <v>-8.130000000000001</v>
       </c>
     </row>
     <row r="18">
@@ -5608,7 +5618,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>-4598.7</v>
+        <v>-5043.04</v>
       </c>
     </row>
     <row r="19">
@@ -5618,7 +5628,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>-383.25</v>
+        <v>-420.28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: monthly data update 2026-07
</commit_message>
<xml_diff>
--- a/data/processed/salary_tracker_uk.xlsx
+++ b/data/processed/salary_tracker_uk.xlsx
@@ -502,7 +502,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B461"/>
+  <dimension ref="A1:B462"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5115,6 +5115,16 @@
       </c>
       <c r="B461" t="n">
         <v>142.1</v>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B462" t="n">
+        <v>142.4</v>
       </c>
     </row>
   </sheetData>
@@ -5457,7 +5467,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-04</t>
+          <t>2026-05</t>
         </is>
       </c>
     </row>
@@ -5468,7 +5478,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>142.1</v>
+        <v>142.4</v>
       </c>
     </row>
     <row r="4">
@@ -5558,7 +5568,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>4746.72</v>
+        <v>4736.72</v>
       </c>
     </row>
     <row r="13">
@@ -5568,7 +5578,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>56956.96</v>
+        <v>56836.96</v>
       </c>
     </row>
     <row r="14">
@@ -5578,7 +5588,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>29.21</v>
+        <v>29.15</v>
       </c>
     </row>
     <row r="15">
@@ -5588,7 +5598,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>8.85</v>
+        <v>9.08</v>
       </c>
     </row>
     <row r="16">
@@ -5608,7 +5618,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>-8.130000000000001</v>
+        <v>-8.33</v>
       </c>
     </row>
     <row r="18">
@@ -5618,7 +5628,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>-5043.04</v>
+        <v>-5163.04</v>
       </c>
     </row>
     <row r="19">
@@ -5628,7 +5638,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>-420.28</v>
+        <v>-430.28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: monthly data update 2026-08
</commit_message>
<xml_diff>
--- a/data/processed/salary_tracker_uk.xlsx
+++ b/data/processed/salary_tracker_uk.xlsx
@@ -502,7 +502,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B462"/>
+  <dimension ref="A1:B463"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5125,6 +5125,16 @@
       </c>
       <c r="B462" t="n">
         <v>142.4</v>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B463" t="n">
+        <v>142.5</v>
       </c>
     </row>
   </sheetData>
@@ -5467,7 +5477,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05</t>
+          <t>2026-06</t>
         </is>
       </c>
     </row>
@@ -5478,7 +5488,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>142.4</v>
+        <v>142.5</v>
       </c>
     </row>
     <row r="4">
@@ -5568,7 +5578,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>4736.72</v>
+        <v>4733.4</v>
       </c>
     </row>
     <row r="13">
@@ -5578,7 +5588,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>56836.96</v>
+        <v>56797.08</v>
       </c>
     </row>
     <row r="14">
@@ -5588,7 +5598,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>29.15</v>
+        <v>29.13</v>
       </c>
     </row>
     <row r="15">
@@ -5598,7 +5608,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>9.08</v>
+        <v>9.16</v>
       </c>
     </row>
     <row r="16">
@@ -5618,7 +5628,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>-8.33</v>
+        <v>-8.390000000000001</v>
       </c>
     </row>
     <row r="18">
@@ -5628,7 +5638,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>-5163.04</v>
+        <v>-5202.92</v>
       </c>
     </row>
     <row r="19">
@@ -5638,7 +5648,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>-430.28</v>
+        <v>-433.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: monthly data update 2026-09
</commit_message>
<xml_diff>
--- a/data/processed/salary_tracker_uk.xlsx
+++ b/data/processed/salary_tracker_uk.xlsx
@@ -502,7 +502,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B463"/>
+  <dimension ref="A1:B464"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5135,6 +5135,16 @@
       </c>
       <c r="B463" t="n">
         <v>142.5</v>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B464" t="n">
+        <v>142.9</v>
       </c>
     </row>
   </sheetData>
@@ -5477,7 +5487,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06</t>
+          <t>2026-07</t>
         </is>
       </c>
     </row>
@@ -5488,7 +5498,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>142.5</v>
+        <v>142.9</v>
       </c>
     </row>
     <row r="4">
@@ -5578,7 +5588,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>4733.4</v>
+        <v>4720.15</v>
       </c>
     </row>
     <row r="13">
@@ -5588,7 +5598,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>56797.08</v>
+        <v>56638.09</v>
       </c>
     </row>
     <row r="14">
@@ -5598,7 +5608,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>29.13</v>
+        <v>29.05</v>
       </c>
     </row>
     <row r="15">
@@ -5608,7 +5618,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>9.16</v>
+        <v>9.470000000000001</v>
       </c>
     </row>
     <row r="16">
@@ -5628,7 +5638,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>-8.390000000000001</v>
+        <v>-8.65</v>
       </c>
     </row>
     <row r="18">
@@ -5638,7 +5648,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>-5202.92</v>
+        <v>-5361.91</v>
       </c>
     </row>
     <row r="19">
@@ -5648,7 +5658,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>-433.6</v>
+        <v>-446.85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>